<commit_message>
finalizado criar e addd conta
</commit_message>
<xml_diff>
--- a/cliente_banco_Tabajara.xlsx
+++ b/cliente_banco_Tabajara.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,11 +451,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>jon</t>
+          <t>asd</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2222</v>
+        <v>112323</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -469,6 +469,30 @@
         <v>400</v>
       </c>
       <c r="F2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>jos</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>22222</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>sal</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" t="n">
+        <v>401</v>
+      </c>
+      <c r="F3" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>